<commit_message>
Atualização automática do Dashboard VBP
</commit_message>
<xml_diff>
--- a/bases_historicas/base_consolidada_06-2026.xlsx
+++ b/bases_historicas/base_consolidada_06-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ125"/>
+  <dimension ref="A1:AY126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,6 +632,46 @@
           <t>%_2026/2025</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>cod_uf</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>produto</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>milhoes_r$</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>uf_regioesnome_uf</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>uf_regioesregiao</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -767,6 +807,30 @@
       <c r="AQ2" t="n">
         <v>-0.1477492356937435</v>
       </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -902,6 +966,30 @@
       <c r="AQ3" t="n">
         <v>-0.144735375026774</v>
       </c>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1037,6 +1125,30 @@
       <c r="AQ4" t="n">
         <v>-0.3046397707586472</v>
       </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1172,6 +1284,30 @@
       <c r="AQ5" t="n">
         <v>0.04590561817211603</v>
       </c>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1307,6 +1443,30 @@
       <c r="AQ6" t="n">
         <v>-0.07958030437074204</v>
       </c>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1442,6 +1602,30 @@
       <c r="AQ7" t="n">
         <v>-0.3366112925492458</v>
       </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1593,6 +1777,30 @@
       <c r="AQ8" t="n">
         <v>0.01259420521597976</v>
       </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1744,6 +1952,30 @@
       <c r="AQ9" t="n">
         <v>0.09191339116488573</v>
       </c>
+      <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1923,6 +2155,30 @@
       <c r="AQ10" t="n">
         <v>-0.1942989061596975</v>
       </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2058,6 +2314,30 @@
       <c r="AQ11" t="n">
         <v>-0.1117422278449733</v>
       </c>
+      <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2217,6 +2497,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2352,6 +2656,30 @@
       <c r="AQ13" t="n">
         <v>0.08359147039035997</v>
       </c>
+      <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2513,6 +2841,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2648,6 +3000,30 @@
       <c r="AQ15" t="n">
         <v>-0.3614886570807894</v>
       </c>
+      <c r="AR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2789,6 +3165,30 @@
       <c r="AQ16" t="n">
         <v>-1</v>
       </c>
+      <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2924,6 +3324,30 @@
       <c r="AQ17" t="n">
         <v>0.2687244626285463</v>
       </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3059,6 +3483,30 @@
       <c r="AQ18" t="n">
         <v>-0.07110976387488355</v>
       </c>
+      <c r="AR18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3218,6 +3666,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3353,6 +3825,30 @@
       <c r="AQ20" t="n">
         <v>0.03742051884185704</v>
       </c>
+      <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3488,6 +3984,30 @@
       <c r="AQ21" t="n">
         <v>-0.1530049413722474</v>
       </c>
+      <c r="AR21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3623,6 +4143,30 @@
       <c r="AQ22" t="n">
         <v>-0.1734924717057609</v>
       </c>
+      <c r="AR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3758,6 +4302,30 @@
       <c r="AQ23" t="n">
         <v>-0.1692240276811933</v>
       </c>
+      <c r="AR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3961,6 +4529,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4096,6 +4688,30 @@
       <c r="AQ25" t="n">
         <v>-0.03971758425956684</v>
       </c>
+      <c r="AR25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4253,6 +4869,30 @@
       <c r="AQ26" t="n">
         <v>0.03206216685625241</v>
       </c>
+      <c r="AR26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4410,6 +5050,30 @@
       <c r="AQ27" t="n">
         <v>-0.04436079664406711</v>
       </c>
+      <c r="AR27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4567,6 +5231,30 @@
       <c r="AQ28" t="n">
         <v>-0.0742773947458103</v>
       </c>
+      <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4724,6 +5412,30 @@
       <c r="AQ29" t="n">
         <v>-0.04045337327045928</v>
       </c>
+      <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4881,6 +5593,30 @@
       <c r="AQ30" t="n">
         <v>-0.2443135501141886</v>
       </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5038,6 +5774,30 @@
       <c r="AQ31" t="n">
         <v>-0.02954892692782762</v>
       </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5173,6 +5933,30 @@
       <c r="AQ32" t="n">
         <v>-0.0362153892529341</v>
       </c>
+      <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5308,6 +6092,30 @@
       <c r="AQ33" t="n">
         <v>-0.1623046230134449</v>
       </c>
+      <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5443,6 +6251,30 @@
       <c r="AQ34" t="n">
         <v>-0.1308690726229079</v>
       </c>
+      <c r="AR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5578,6 +6410,30 @@
       <c r="AQ35" t="n">
         <v>-0.3043837685703291</v>
       </c>
+      <c r="AR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5713,6 +6569,30 @@
       <c r="AQ36" t="n">
         <v>0.02251180080502158</v>
       </c>
+      <c r="AR36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5848,6 +6728,30 @@
       <c r="AQ37" t="n">
         <v>-0.1207206783576501</v>
       </c>
+      <c r="AR37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5983,6 +6887,30 @@
       <c r="AQ38" t="n">
         <v>-0.4315494033687179</v>
       </c>
+      <c r="AR38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6134,6 +7062,30 @@
       <c r="AQ39" t="n">
         <v>-0.01612436888096913</v>
       </c>
+      <c r="AR39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6285,6 +7237,30 @@
       <c r="AQ40" t="n">
         <v>0.07540445855671774</v>
       </c>
+      <c r="AR40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6464,6 +7440,30 @@
       <c r="AQ41" t="n">
         <v>-0.2548646391271715</v>
       </c>
+      <c r="AR41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6599,6 +7599,30 @@
       <c r="AQ42" t="n">
         <v>-0.08156137571914579</v>
       </c>
+      <c r="AR42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6758,6 +7782,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6893,6 +7941,30 @@
       <c r="AQ44" t="n">
         <v>0.1302470662615371</v>
       </c>
+      <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7054,6 +8126,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7189,6 +8285,30 @@
       <c r="AQ46" t="n">
         <v>-0.3761218357052035</v>
       </c>
+      <c r="AR46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7330,6 +8450,30 @@
       <c r="AQ47" t="n">
         <v>-1</v>
       </c>
+      <c r="AR47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7465,6 +8609,30 @@
       <c r="AQ48" t="n">
         <v>0.2108688733318391</v>
       </c>
+      <c r="AR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7600,6 +8768,30 @@
       <c r="AQ49" t="n">
         <v>-0.06849971080666761</v>
       </c>
+      <c r="AR49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7759,6 +8951,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7894,6 +9110,30 @@
       <c r="AQ51" t="n">
         <v>0.01186367562223789</v>
       </c>
+      <c r="AR51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8029,6 +9269,30 @@
       <c r="AQ52" t="n">
         <v>-0.1406601173444304</v>
       </c>
+      <c r="AR52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8164,6 +9428,30 @@
       <c r="AQ53" t="n">
         <v>-0.1726922586413705</v>
       </c>
+      <c r="AR53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8299,6 +9587,30 @@
       <c r="AQ54" t="n">
         <v>-0.1280095322180227</v>
       </c>
+      <c r="AR54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8502,6 +9814,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8637,6 +9973,30 @@
       <c r="AQ56" t="n">
         <v>-0.05078890261913405</v>
       </c>
+      <c r="AR56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8794,6 +10154,30 @@
       <c r="AQ57" t="n">
         <v>0.05556533801765928</v>
       </c>
+      <c r="AR57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8951,6 +10335,30 @@
       <c r="AQ58" t="n">
         <v>-0.1037870962900198</v>
       </c>
+      <c r="AR58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9108,6 +10516,30 @@
       <c r="AQ59" t="n">
         <v>-0.08538514697789512</v>
       </c>
+      <c r="AR59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9265,6 +10697,30 @@
       <c r="AQ60" t="n">
         <v>-0.05135885130628592</v>
       </c>
+      <c r="AR60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9422,6 +10878,30 @@
       <c r="AQ61" t="n">
         <v>-0.1555238142007428</v>
       </c>
+      <c r="AR61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -9579,6 +11059,30 @@
       <c r="AQ62" t="n">
         <v>-0.02591193701644889</v>
       </c>
+      <c r="AR62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9714,6 +11218,30 @@
       <c r="AQ63" t="n">
         <v>-0.04222100797271311</v>
       </c>
+      <c r="AR63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9849,6 +11377,30 @@
       <c r="AQ64" t="n">
         <v>-0.1556386994536925</v>
       </c>
+      <c r="AR64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9984,6 +11536,30 @@
       <c r="AQ65" t="n">
         <v>-0.1346345667197874</v>
       </c>
+      <c r="AR65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10119,6 +11695,30 @@
       <c r="AQ66" t="n">
         <v>-0.3108405327089913</v>
       </c>
+      <c r="AR66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -10254,6 +11854,30 @@
       <c r="AQ67" t="n">
         <v>0.04512213111577457</v>
       </c>
+      <c r="AR67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -10389,6 +12013,30 @@
       <c r="AQ68" t="n">
         <v>-0.04832591019083032</v>
       </c>
+      <c r="AR68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -10524,6 +12172,30 @@
       <c r="AQ69" t="n">
         <v>-0.5203184280731676</v>
       </c>
+      <c r="AR69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10675,6 +12347,30 @@
       <c r="AQ70" t="n">
         <v>-0.03134259812820295</v>
       </c>
+      <c r="AR70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10826,6 +12522,30 @@
       <c r="AQ71" t="n">
         <v>0.05427561125353297</v>
       </c>
+      <c r="AR71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -11005,6 +12725,30 @@
       <c r="AQ72" t="n">
         <v>-0.2546658397561753</v>
       </c>
+      <c r="AR72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -11140,6 +12884,30 @@
       <c r="AQ73" t="n">
         <v>-0.07159360050667773</v>
       </c>
+      <c r="AR73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11299,6 +13067,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11434,6 +13226,30 @@
       <c r="AQ75" t="n">
         <v>0.1416159968591346</v>
       </c>
+      <c r="AR75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -11595,6 +13411,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -11730,6 +13570,30 @@
       <c r="AQ77" t="n">
         <v>-0.3664835448960276</v>
       </c>
+      <c r="AR77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -11869,6 +13733,30 @@
       <c r="AQ78" t="n">
         <v>-0.2056620933699921</v>
       </c>
+      <c r="AR78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -12004,6 +13892,30 @@
       <c r="AQ79" t="n">
         <v>0.1695079030725881</v>
       </c>
+      <c r="AR79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -12139,6 +14051,30 @@
       <c r="AQ80" t="n">
         <v>-0.04530497319769411</v>
       </c>
+      <c r="AR80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -12298,6 +14234,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -12433,6 +14393,30 @@
       <c r="AQ82" t="n">
         <v>0.00516554058134977</v>
       </c>
+      <c r="AR82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -12568,6 +14552,30 @@
       <c r="AQ83" t="n">
         <v>-0.08283159988181688</v>
       </c>
+      <c r="AR83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -12703,6 +14711,30 @@
       <c r="AQ84" t="n">
         <v>-0.1970892292043684</v>
       </c>
+      <c r="AR84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -12838,6 +14870,30 @@
       <c r="AQ85" t="n">
         <v>-0.08850027086830814</v>
       </c>
+      <c r="AR85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13041,6 +15097,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13176,6 +15256,30 @@
       <c r="AQ87" t="n">
         <v>-0.04825491394547021</v>
       </c>
+      <c r="AR87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -13333,6 +15437,30 @@
       <c r="AQ88" t="n">
         <v>0.0739688801663192</v>
       </c>
+      <c r="AR88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13490,6 +15618,30 @@
       <c r="AQ89" t="n">
         <v>-0.1281021341327407</v>
       </c>
+      <c r="AR89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -13647,6 +15799,30 @@
       <c r="AQ90" t="n">
         <v>-0.09961898096106248</v>
       </c>
+      <c r="AR90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13804,6 +15980,30 @@
       <c r="AQ91" t="n">
         <v>-0.05806958125620243</v>
       </c>
+      <c r="AR91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -13961,6 +16161,30 @@
       <c r="AQ92" t="n">
         <v>-0.09845933605775981</v>
       </c>
+      <c r="AR92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -14118,6 +16342,30 @@
       <c r="AQ93" t="n">
         <v>-0.02103966684572445</v>
       </c>
+      <c r="AR93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14253,6 +16501,30 @@
       <c r="AQ94" t="n">
         <v>-0.03870955817030419</v>
       </c>
+      <c r="AR94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -14388,6 +16660,30 @@
       <c r="AQ95" t="n">
         <v>-0.1168929827771792</v>
       </c>
+      <c r="AR95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -14523,6 +16819,30 @@
       <c r="AQ96" t="n">
         <v>-0.1352829990226698</v>
       </c>
+      <c r="AR96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -14658,6 +16978,30 @@
       <c r="AQ97" t="n">
         <v>-0.3044354858732528</v>
       </c>
+      <c r="AR97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -14793,6 +17137,30 @@
       <c r="AQ98" t="n">
         <v>0.03974687842150981</v>
       </c>
+      <c r="AR98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -14928,6 +17296,30 @@
       <c r="AQ99" t="n">
         <v>0.006952748022160948</v>
       </c>
+      <c r="AR99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -15063,6 +17455,30 @@
       <c r="AQ100" t="n">
         <v>-0.5470944717349852</v>
       </c>
+      <c r="AR100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15214,6 +17630,30 @@
       <c r="AQ101" t="n">
         <v>-0.05528612197641947</v>
       </c>
+      <c r="AR101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -15365,6 +17805,30 @@
       <c r="AQ102" t="n">
         <v>0.02189291393770132</v>
       </c>
+      <c r="AR102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -15544,6 +18008,30 @@
       <c r="AQ103" t="n">
         <v>-0.2565969483826996</v>
       </c>
+      <c r="AR103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -15679,6 +18167,30 @@
       <c r="AQ104" t="n">
         <v>-0.07531577390127897</v>
       </c>
+      <c r="AR104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -15838,6 +18350,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -15973,6 +18509,30 @@
       <c r="AQ106" t="n">
         <v>0.1174433643050921</v>
       </c>
+      <c r="AR106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -16134,6 +18694,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -16269,6 +18853,30 @@
       <c r="AQ108" t="n">
         <v>-0.3653811701925</v>
       </c>
+      <c r="AR108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -16408,6 +19016,30 @@
       <c r="AQ109" t="n">
         <v>-0.2038406459359604</v>
       </c>
+      <c r="AR109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -16543,6 +19175,30 @@
       <c r="AQ110" t="n">
         <v>0.1247402087805252</v>
       </c>
+      <c r="AR110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -16678,6 +19334,30 @@
       <c r="AQ111" t="n">
         <v>-0.05435766796337427</v>
       </c>
+      <c r="AR111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -16837,6 +19517,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -16972,6 +19676,30 @@
       <c r="AQ113" t="n">
         <v>-0.004969953223310508</v>
       </c>
+      <c r="AR113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -17107,6 +19835,30 @@
       <c r="AQ114" t="n">
         <v>-0.01979222948205006</v>
       </c>
+      <c r="AR114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -17242,6 +19994,30 @@
       <c r="AQ115" t="n">
         <v>-0.1894961932674049</v>
       </c>
+      <c r="AR115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -17377,6 +20153,30 @@
       <c r="AQ116" t="n">
         <v>-0.09165895556976034</v>
       </c>
+      <c r="AR116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -17580,6 +20380,30 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -17715,6 +20539,30 @@
       <c r="AQ118" t="n">
         <v>-0.05496713936387976</v>
       </c>
+      <c r="AR118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -17872,6 +20720,30 @@
       <c r="AQ119" t="n">
         <v>0.08818536138406108</v>
       </c>
+      <c r="AR119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -18029,6 +20901,30 @@
       <c r="AQ120" t="n">
         <v>-0.1667073764313325</v>
       </c>
+      <c r="AR120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -18186,6 +21082,30 @@
       <c r="AQ121" t="n">
         <v>-0.1043542569700028</v>
       </c>
+      <c r="AR121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -18343,6 +21263,30 @@
       <c r="AQ122" t="n">
         <v>-0.05472336231550468</v>
       </c>
+      <c r="AR122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -18500,6 +21444,30 @@
       <c r="AQ123" t="n">
         <v>-0.07951467522900968</v>
       </c>
+      <c r="AR123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -18657,6 +21625,30 @@
       <c r="AQ124" t="n">
         <v>-0.01920298720380165</v>
       </c>
+      <c r="AR124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -18791,6 +21783,197 @@
       </c>
       <c r="AQ125" t="n">
         <v>-0.04242337832015575</v>
+      </c>
+      <c r="AR125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026 - 04</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0</v>
+      </c>
+      <c r="J126" t="n">
+        <v>0</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
+        <v>0</v>
+      </c>
+      <c r="S126" t="n">
+        <v>0</v>
+      </c>
+      <c r="T126" t="n">
+        <v>0</v>
+      </c>
+      <c r="U126" t="n">
+        <v>0</v>
+      </c>
+      <c r="V126" t="n">
+        <v>0</v>
+      </c>
+      <c r="W126" t="n">
+        <v>0</v>
+      </c>
+      <c r="X126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR126" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="AS126" t="inlineStr">
+        <is>
+          <t>ALGODÃO</t>
+        </is>
+      </c>
+      <c r="AT126" t="n">
+        <v>2018</v>
+      </c>
+      <c r="AU126" t="n">
+        <v>91430521.9375</v>
+      </c>
+      <c r="AV126" t="n">
+        <v>91.43049999999999</v>
+      </c>
+      <c r="AW126" t="inlineStr">
+        <is>
+          <t>LAVOURAS</t>
+        </is>
+      </c>
+      <c r="AX126" t="inlineStr">
+        <is>
+          <t>RONDÔNIA</t>
+        </is>
+      </c>
+      <c r="AY126" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>